<commit_message>
Acrescentei uma coluna a mais pra centralizar a logo na planilha final
</commit_message>
<xml_diff>
--- a/modelos/OdP's de cada funcionário.xlsx
+++ b/modelos/OdP's de cada funcionário.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EECA012-FB6A-4718-9F39-15D5CDC62579}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1011B5D-9C9D-464D-9055-94FADC940A79}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,22 +83,26 @@
       <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="30"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -106,11 +110,13 @@
       <sz val="14"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -128,7 +134,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -238,31 +244,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -290,14 +276,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -307,6 +285,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,28 +510,29 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z6"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" customWidth="1"/>
-    <col min="7" max="7" width="29.140625" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" customWidth="1"/>
-    <col min="9" max="9" width="19.85546875" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" customWidth="1"/>
-    <col min="11" max="11" width="75.7109375" customWidth="1"/>
+    <col min="1" max="1" width="1.42578125" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="19.5703125" customWidth="1"/>
+    <col min="8" max="8" width="29.140625" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" customWidth="1"/>
+    <col min="11" max="11" width="21.5703125" customWidth="1"/>
+    <col min="12" max="12" width="75.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="11"/>
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="18"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="10"/>
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
       <c r="F1" s="10"/>
@@ -559,10 +541,11 @@
       <c r="I1" s="10"/>
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
     </row>
-    <row r="2" spans="1:26" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="12"/>
-      <c r="B2" s="10"/>
+    <row r="2" spans="1:27" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
@@ -572,74 +555,77 @@
       <c r="I2" s="10"/>
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
     </row>
-    <row r="3" spans="1:26" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="7" t="s">
+    <row r="3" spans="1:27" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="8"/>
+      <c r="E3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="9"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="8" t="s">
+      <c r="F3" s="9"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="8"/>
+      <c r="J3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="9"/>
-      <c r="K3" s="17"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="13"/>
     </row>
-    <row r="4" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14"/>
+    <row r="4" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="18"/>
       <c r="B4" s="18"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="20"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
       <c r="F4" s="16"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="20"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
       <c r="K4" s="16"/>
+      <c r="L4" s="12"/>
     </row>
-    <row r="5" spans="1:26" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="14"/>
-      <c r="B5" s="6" t="s">
+    <row r="5" spans="1:27" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
@@ -649,24 +635,25 @@
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
-      <c r="V5" s="4"/>
+      <c r="V5" s="3"/>
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
       <c r="Y5" s="4"/>
       <c r="Z5" s="4"/>
+      <c r="AA5" s="4"/>
     </row>
-    <row r="6" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="K6" s="5"/>
+    <row r="6" spans="1:27" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L6" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B1:K2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="C1:L2"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="A3:B5"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>